<commit_message>
[brazil-only] Refresh Brazil news and import premium
</commit_message>
<xml_diff>
--- a/reports/2026/07/Sugar News 2026-07-26.xlsx
+++ b/reports/2026/07/Sugar News 2026-07-26.xlsx
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="55" customWidth="1" style="2" min="2" max="2"/>
@@ -508,17 +508,17 @@
     <row r="2" ht="180" customHeight="1" s="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>印度</t>
+          <t>巴西</t>
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>simplywall.st消息涉及印度糖业运行变化。该事项对食糖供应、需求或价格的影响仍需结合后续政策、产量和贸易数据继续跟踪。来源：simplywall.st（https://news.google.com/rss/articles/CBMi-gFBVV95cUxPNjhaWldCbjFQNVV3cTRublJKVEUxSlRMNllDX0JJdkNaUGxTcngycEtUX1BJSHNWZXo5NkhqNkpjdUpVcGRsT05UeXU4SEh6b0MyclFNb1pzaVctTmVvdUFqaHc2cmVOU1Z1SEJXWXZLTlNlVVFUUmxCYmZ6d1NFdTZ5V2l2MHFSckc1YnA3YXNITUF1a0syWElibXMtOWxXU2Rka2xHam9aT2dPNmt2R1ZGRzhpRHRvVG1VT1o1bzJXb25rRkRqTWIzNWo3TWM4X0RVWHBwZ0tvNHMzQ0ttQ0RLWHFZcGJLVnIycGFEVndEUTUzSmQyNzhR0gH_AUFVX3lxTFB0WmZVZlFzNEwxYXpGamx2WjJFZkVCSXRmOEVBNkRXWkVUWG5XcUphbi12UldnRWNSR2VTVFAwb2dRb25iUy05RkZyd2pLN1lNNzhsMTFnQnNpSlpobFoyYVJyMVB3Y1hWSUx2bVYzRTJiMDNXUlZfSk5fWDNBSFNoV2hjdG9neHpValBVU3FLeWF2RG1CSTU2cDFLcndYdmJXU3Z6d1A1dWZaVjB2RGFzMFJSNnhvaFpiZ3JMMFdnWDg4XzRPa05lYjZmZVd2M0JRbFRTTnJNWHR5UFNiSEVNRnFNclVjSHBOVzRJTG1BaWR3eVpMclMzOWRuZFlvTQ?oc=5）</t>
+          <t>Banco do Nordeste旗下ETENE预计，巴西东北部2026/27榨季甘蔗产量将增长3.7%，其中种植面积增加1.3%、单产提高2.3%；区域糖产量预计达到363万吨，同比增加10.3%。甘蔗供应和制糖产出同步增长将增加巴西可用糖源，对糖价形成利空影响。来源：Banco do Nordeste（https://www.bnb.gov.br/web/guest/imprensa/noticias/-/asset_publisher/QGdgGhxvRtMv/content/produ%C3%A7%C3%A3o-de-a%C3%A7%C3%BAcar-no-nordeste-deve-se-recuperar-com-mais-oferta-de-cana-e-avan%C3%A7o-tecnol%C3%B3gico-no-campo/44540）</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>中性：该信息需要继续跟踪，短期对当期糖产量和出口量的直接影响有限。</t>
+          <t>利空：巴西东北部甘蔗和食糖产量预期增加，将扩大区域糖源供应并对糖价形成压力。</t>
         </is>
       </c>
     </row>
@@ -530,7 +530,7 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>ANTARA News消息涉及印度尼西亚乙醇、糖蜜或糖料分流安排。若甘蔗、糖蜜或糖浆更多流向制醇，可能减少制糖供应；反之则可能增加食糖产出。来源：ANTARA News（https://news.google.com/rss/articles/CBMipgFBVV95cUxOYW5FTDRyWERiOGh5VGN2dkI0NlJzTW5Ia1JRclJxZDBzLWFaOXpwSS1qS3NyamFobWFrUlQxNGFqQU96VjhzMUhyZ0xFa0hJTV9QcHlGN1dvRU16MVpvWFlVcHZQbURnOVdnR2tZSVNaUHFxc0hYTC1ybzdacFVNNlNyWXFDa0R3UmJ5R2RiNTRGeUlRNWFmQ1puUVFCdmNsSDBNcWlR0gGrAUFVX3lxTE1YdG9Gb0N5TmhyaExSNldlZkZhSHBpNXJoV25iSDNMc2hTWmNKR3V3VjNLMDd3ZW1nTWJYaTdqNWZYcFpkOEdaSGFXNmMzeTNWejh3WTZBUl9pcHFHTTdDazgzM0p2SXYxTW0weVN3S2lnUURnOVAtRTJ2MWt5Q1VUUFlqS2R3RG5ZdmRVblk4UXctV0tra0tzVEtQcnE4VUp4RFBTUzgtY0RLZw?oc=5）</t>
+          <t>simplywall.st消息涉及印度糖业运行变化。该事项对食糖供应、需求或价格的影响仍需结合后续政策、产量和贸易数据继续跟踪。来源：simplywall.st（https://news.google.com/rss/articles/CBMi-gFBVV95cUxPNjhaWldCbjFQNVV3cTRublJKVEUxSlRMNllDX0JJdkNaUGxTcngycEtUX1BJSHNWZXo5NkhqNkpjdUpVcGRsT05UeXU4SEh6b0MyclFNb1pzaVctTmVvdUFqaHc2cmVOU1Z1SEJXWXZLTlNlVVFUUmxCYmZ6d1NFdTZ5V2l2MHFSckc1YnA3YXNITUF1a0syWElibXMtOWxXU2Rka2xHam9aT2dPNmt2R1ZGRzhpRHRvVG1VT1o1bzJXb25rRkRqTWIzNWo3TWM4X0RVWHBwZ0tvNHMzQ0ttQ0RLWHFZcGJLVnIycGFEVndEUTUzSmQyNzhR0gH_AUFVX3lxTFB0WmZVZlFzNEwxYXpGamx2WjJFZkVCSXRmOEVBNkRXWkVUWG5XcUphbi12UldnRWNSR2VTVFAwb2dRb25iUy05RkZyd2pLN1lNNzhsMTFnQnNpSlpobFoyYVJyMVB3Y1hWSUx2bVYzRTJiMDNXUlZfSk5fWDNBSFNoV2hjdG9neHpValBVU3FLeWF2RG1CSTU2cDFLcndYdmJXU3Z6d1A1dWZaVjB2RGFzMFJSNnhvaFpiZ3JMMFdnWDg4XzRPa05lYjZmZVd2M0JRbFRTTnJNWHR5UFNiSEVNRnFNclVjSHBOVzRJTG1BaWR3eVpMclMzOWRuZFlvTQ?oc=5）</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
@@ -547,44 +547,61 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
+          <t>ANTARA News消息涉及印度尼西亚乙醇、糖蜜或糖料分流安排。若甘蔗、糖蜜或糖浆更多流向制醇，可能减少制糖供应；反之则可能增加食糖产出。来源：ANTARA News（https://news.google.com/rss/articles/CBMipgFBVV95cUxOYW5FTDRyWERiOGh5VGN2dkI0NlJzTW5Ia1JRclJxZDBzLWFaOXpwSS1qS3NyamFobWFrUlQxNGFqQU96VjhzMUhyZ0xFa0hJTV9QcHlGN1dvRU16MVpvWFlVcHZQbURnOVdnR2tZSVNaUHFxc0hYTC1ybzdacFVNNlNyWXFDa0R3UmJ5R2RiNTRGeUlRNWFmQ1puUVFCdmNsSDBNcWlR0gGrAUFVX3lxTE1YdG9Gb0N5TmhyaExSNldlZkZhSHBpNXJoV25iSDNMc2hTWmNKR3V3VjNLMDd3ZW1nTWJYaTdqNWZYcFpkOEdaSGFXNmMzeTNWejh3WTZBUl9pcHFHTTdDazgzM0p2SXYxTW0weVN3S2lnUURnOVAtRTJ2MWt5Q1VUUFlqS2R3RG5ZdmRVblk4UXctV0tra0tzVEtQcnE4VUp4RFBTUzgtY0RLZw?oc=5）</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>中性：该信息需要继续跟踪，短期对当期糖产量和出口量的直接影响有限。</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="180" customHeight="1" s="2">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>印度</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
           <t>The Economic Times消息涉及印度糖业运行变化。该事项对食糖供应、需求或价格的影响仍需结合后续政策、产量和贸易数据继续跟踪。来源：The Economic Times（https://news.google.com/rss/articles/CBMiowJBVV95cUxQbWt4LXZjZ2FBdFRYMmtjNXhmVWJ4ZEhLT2VRbU1pVEhiazNfX04yLW1sTGVDUEU3WTZUTC1XdlhjWU9sLXFuTC1Mb0NTQ2R1YXhLV3FXT21NVWZwNnplblJDWGN2NG1HcHRJME5Dcl8xQ0k2NHV4QkZGS1RpVHYtd3BfZnR4b3R4WmN5ZGV2aWpISWU0cXFhMUhpb2FJOHdyYXVfaDZLZHdYeWJQaXZneGg3WHFJLWZBVU4zQjYtT1NGNG9WVlVXQ05kbGhEN1RKQllIWW51VVVOazVaMnQzMHVJMjUyY0tVdUhneU4wbm0wcE9uRWVENHNsX1NwMmUtbW42enFDR0tzQ2dDQmRiSkpsa3Y0eVpMMkloMDVHUlhyLTTSAaMCQVVfeXFMUG1reC12Y2dhQXRUWDJrYzV4ZlVieGRIS09lUW1NaVRIYmszX19OMi1tbExlQ1BFN1k2VEwtV3ZYY1lPbC1xbkwtTG9DU0NkdWF4S1dxV09tTVVmcDZ6ZW5SQ1hjdjRtR3B0STBOQ3JfMUNJNjR1eEJGRktUaVR2LXdwX2Z0eG90eFpjeWRldmlqSEllNHFxYTFIaW9hSTh3cmF1X2g2S2R3WHliUGl2Z3hoN1hxSS1mQVVOM0I2LU9TRjRvVlZVV0NOZGxoRDdUSkJZSFludVVVTms1WjJ0MzB1STI1MmNLVXVIZ3lOMG5tMHBPbkVlRDRzbF9TcDJlLW1uNnpxQ0dLc0NnQ0JkYkpKbGt2NHlaTDJJaDA1R1JYci00?oc=5）</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>中性：该信息需要继续跟踪，短期对当期糖产量和出口量的直接影响有限。</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="114.2" customHeight="1" s="2">
-      <c r="A5" s="3" t="inlineStr">
+    <row r="6" ht="114.2" customHeight="1" s="2">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t>泰国</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>泰国气象局预报（2026-07-26），乌隆他尼、彭世洛、北碧、猜纳等主要甘蔗产区预计出现雷阵雨并伴有局地大雨。当前处于甘蔗生长阶段，强降雨、雷阵雨以及预报大雨均有利于补充产区土壤水分，促进甘蔗生长和单产形成，提高后期甘蔗及食糖产量预期。来源：泰国气象局（https://tmd.go.th/en/forecast/daily）</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C6" s="4" t="inlineStr">
         <is>
           <t>利空：甘蔗生长阶段的降雨有利于补充土壤水分、改善墒情并促进甘蔗生长和单产形成，从而增加未来甘蔗及食糖供应预期，因此利空糖价。</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="118.05" customHeight="1" s="2">
-      <c r="A6" s="3" t="inlineStr">
+    <row r="7" ht="118.05" customHeight="1" s="2">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>中国</t>
         </is>
       </c>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>已完成中国食糖、甘蔗、甜菜糖、进口、库存、现货价格和主产区天气等重点方向监测，未发现符合收录标准的新增重要糖业事件。该结果仅表示本次公开来源检索没有可发布的新事件，不代表中国食糖供需或价格没有变化。来源：Sugar News中国糖业每日监测日志（https://github.com/lishi2626/sugar-news/actions）</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>中性：本次监测未发现足以改变中国食糖供需、库存、进口或价格预期的新增公开信息。</t>
         </is>

</xml_diff>

<commit_message>
Tighten Sugar News summary quality rules
</commit_message>
<xml_diff>
--- a/reports/2026/07/Sugar News 2026-07-26.xlsx
+++ b/reports/2026/07/Sugar News 2026-07-26.xlsx
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="55" customWidth="1" style="2" min="2" max="2"/>
@@ -522,88 +522,54 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="180" customHeight="1" s="2">
+    <row r="3" ht="114.2" customHeight="1" s="2">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>印度</t>
+          <t>泰国</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>simplywall.st消息涉及印度糖业运行变化。该事项对食糖供应、需求或价格的影响仍需结合后续政策、产量和贸易数据继续跟踪。来源：simplywall.st（https://news.google.com/rss/articles/CBMi-gFBVV95cUxPNjhaWldCbjFQNVV3cTRublJKVEUxSlRMNllDX0JJdkNaUGxTcngycEtUX1BJSHNWZXo5NkhqNkpjdUpVcGRsT05UeXU4SEh6b0MyclFNb1pzaVctTmVvdUFqaHc2cmVOU1Z1SEJXWXZLTlNlVVFUUmxCYmZ6d1NFdTZ5V2l2MHFSckc1YnA3YXNITUF1a0syWElibXMtOWxXU2Rka2xHam9aT2dPNmt2R1ZGRzhpRHRvVG1VT1o1bzJXb25rRkRqTWIzNWo3TWM4X0RVWHBwZ0tvNHMzQ0ttQ0RLWHFZcGJLVnIycGFEVndEUTUzSmQyNzhR0gH_AUFVX3lxTFB0WmZVZlFzNEwxYXpGamx2WjJFZkVCSXRmOEVBNkRXWkVUWG5XcUphbi12UldnRWNSR2VTVFAwb2dRb25iUy05RkZyd2pLN1lNNzhsMTFnQnNpSlpobFoyYVJyMVB3Y1hWSUx2bVYzRTJiMDNXUlZfSk5fWDNBSFNoV2hjdG9neHpValBVU3FLeWF2RG1CSTU2cDFLcndYdmJXU3Z6d1A1dWZaVjB2RGFzMFJSNnhvaFpiZ3JMMFdnWDg4XzRPa05lYjZmZVd2M0JRbFRTTnJNWHR5UFNiSEVNRnFNclVjSHBOVzRJTG1BaWR3eVpMclMzOWRuZFlvTQ?oc=5）</t>
+          <t>泰国气象局预报（2026-07-26），乌隆他尼、彭世洛、北碧、猜纳等主要甘蔗产区预计出现雷阵雨并伴有局地大雨。当前处于甘蔗生长阶段，强降雨、雷阵雨以及预报大雨均有利于补充产区土壤水分，促进甘蔗生长和单产形成，提高后期甘蔗及食糖产量预期。来源：泰国气象局（https://tmd.go.th/en/forecast/daily）</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>中性：该信息需要继续跟踪，短期对当期糖产量和出口量的直接影响有限。</t>
+          <t>利空：甘蔗生长阶段的降雨有利于补充土壤水分、改善墒情并促进甘蔗生长和单产形成，从而增加未来甘蔗及食糖供应预期，因此利空糖价。</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="180" customHeight="1" s="2">
+    <row r="4" ht="118.05" customHeight="1" s="2">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>印度</t>
+          <t>中国</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>ANTARA News消息涉及印度尼西亚乙醇、糖蜜或糖料分流安排。若甘蔗、糖蜜或糖浆更多流向制醇，可能减少制糖供应；反之则可能增加食糖产出。来源：ANTARA News（https://news.google.com/rss/articles/CBMipgFBVV95cUxOYW5FTDRyWERiOGh5VGN2dkI0NlJzTW5Ia1JRclJxZDBzLWFaOXpwSS1qS3NyamFobWFrUlQxNGFqQU96VjhzMUhyZ0xFa0hJTV9QcHlGN1dvRU16MVpvWFlVcHZQbURnOVdnR2tZSVNaUHFxc0hYTC1ybzdacFVNNlNyWXFDa0R3UmJ5R2RiNTRGeUlRNWFmQ1puUVFCdmNsSDBNcWlR0gGrAUFVX3lxTE1YdG9Gb0N5TmhyaExSNldlZkZhSHBpNXJoV25iSDNMc2hTWmNKR3V3VjNLMDd3ZW1nTWJYaTdqNWZYcFpkOEdaSGFXNmMzeTNWejh3WTZBUl9pcHFHTTdDazgzM0p2SXYxTW0weVN3S2lnUURnOVAtRTJ2MWt5Q1VUUFlqS2R3RG5ZdmRVblk4UXctV0tra0tzVEtQcnE4VUp4RFBTUzgtY0RLZw?oc=5）</t>
+          <t>已完成中国食糖、甘蔗、甜菜糖、进口、库存、现货价格和主产区天气等重点方向监测，未发现符合收录标准的新增重要糖业事件。该结果仅表示本次公开来源检索没有可发布的新事件，不代表中国食糖供需或价格没有变化。来源：Sugar News中国糖业每日监测日志（https://github.com/lishi2626/sugar-news/actions）</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>中性：该信息需要继续跟踪，短期对当期糖产量和出口量的直接影响有限。</t>
+          <t>中性：本次监测未发现足以改变中国食糖供需、库存、进口或价格预期的新增公开信息。</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="180" customHeight="1" s="2">
+    <row r="5" ht="173.05" customHeight="1" s="2">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>印度</t>
+          <t>印度尼西亚</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>The Economic Times消息涉及印度糖业运行变化。该事项对食糖供应、需求或价格的影响仍需结合后续政策、产量和贸易数据继续跟踪。来源：The Economic Times（https://news.google.com/rss/articles/CBMiowJBVV95cUxQbWt4LXZjZ2FBdFRYMmtjNXhmVWJ4ZEhLT2VRbU1pVEhiazNfX04yLW1sTGVDUEU3WTZUTC1XdlhjWU9sLXFuTC1Mb0NTQ2R1YXhLV3FXT21NVWZwNnplblJDWGN2NG1HcHRJME5Dcl8xQ0k2NHV4QkZGS1RpVHYtd3BfZnR4b3R4WmN5ZGV2aWpISWU0cXFhMUhpb2FJOHdyYXVfaDZLZHdYeWJQaXZneGg3WHFJLWZBVU4zQjYtT1NGNG9WVlVXQ05kbGhEN1RKQllIWW51VVVOazVaMnQzMHVJMjUyY0tVdUhneU4wbm0wcE9uRWVENHNsX1NwMmUtbW42enFDR0tzQ2dDQmRiSkpsa3Y0eVpMMkloMDVHUlhyLTTSAaMCQVVfeXFMUG1reC12Y2dhQXRUWDJrYzV4ZlVieGRIS09lUW1NaVRIYmszX19OMi1tbExlQ1BFN1k2VEwtV3ZYY1lPbC1xbkwtTG9DU0NkdWF4S1dxV09tTVVmcDZ6ZW5SQ1hjdjRtR3B0STBOQ3JfMUNJNjR1eEJGRktUaVR2LXdwX2Z0eG90eFpjeWRldmlqSEllNHFxYTFIaW9hSTh3cmF1X2g2S2R3WHliUGl2Z3hoN1hxSS1mQVVOM0I2LU9TRjRvVlZVV0NOZGxoRDdUSkJZSFludVVVTms1WjJ0MzB1STI1MmNLVXVIZ3lOMG5tMHBPbkVlRDRzbF9TcDJlLW1uNnpxQ0dLc0NnQ0JkYkpKbGt2NHlaTDJJaDA1R1JYci00?oc=5）</t>
+          <t>CORE Indonesia经济学家Eliza Mardian表示，印尼每年约生产190万吨糖蜜，其中约90万吨已被利用，仍有约100万吨可用于生物乙醇生产。糖蜜转向燃料级乙醇会提高甘蔗副产品的制醇需求，但印尼燃料级乙醇年产量目前约2.6万千升、全国E10和E20仍需配套投资，短期对食糖供需影响偏中性。来源：ANTARA News（https://en.antaranews.com/news/424096/indonesia-has-1-million-tons-of-molasses-for-bioethanol-economist）</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>中性：该信息需要继续跟踪，短期对当期糖产量和出口量的直接影响有限。</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="114.2" customHeight="1" s="2">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>泰国</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>泰国气象局预报（2026-07-26），乌隆他尼、彭世洛、北碧、猜纳等主要甘蔗产区预计出现雷阵雨并伴有局地大雨。当前处于甘蔗生长阶段，强降雨、雷阵雨以及预报大雨均有利于补充产区土壤水分，促进甘蔗生长和单产形成，提高后期甘蔗及食糖产量预期。来源：泰国气象局（https://tmd.go.th/en/forecast/daily）</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>利空：甘蔗生长阶段的降雨有利于补充土壤水分、改善墒情并促进甘蔗生长和单产形成，从而增加未来甘蔗及食糖供应预期，因此利空糖价。</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="118.05" customHeight="1" s="2">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t>中国</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>已完成中国食糖、甘蔗、甜菜糖、进口、库存、现货价格和主产区天气等重点方向监测，未发现符合收录标准的新增重要糖业事件。该结果仅表示本次公开来源检索没有可发布的新事件，不代表中国食糖供需或价格没有变化。来源：Sugar News中国糖业每日监测日志（https://github.com/lishi2626/sugar-news/actions）</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>中性：本次监测未发现足以改变中国食糖供需、库存、进口或价格预期的新增公开信息。</t>
+          <t>中性：糖蜜潜在制醇量较大，但燃料级乙醇产能和掺混政策仍待投资落地，短期不直接改变区域食糖供应。</t>
         </is>
       </c>
     </row>

</xml_diff>